<commit_message>
ADR line: utilisation (stays per listing) test pre-registered and run — fails the line everywhere, NA in-sample only and pointing to persistence; lap-only residual scenario added beside the base (4Q26 $171.71, on the Street); design addendum on at-or-below-Street constructions
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model/ABNB_official_model.xlsx
+++ b/model/ABNB_official_model.xlsx
@@ -787,7 +787,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'ADR_Engine'!$O$129:$AD$129</f>
+              <f>'ADR_Engine'!$O$130:$AD$130</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -818,7 +818,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'ADR_Engine'!$O$130:$AD$130</f>
+              <f>'ADR_Engine'!$O$131:$AD$131</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -906,7 +906,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'ADR_Engine'!$O$131:$AD$131</f>
+              <f>'ADR_Engine'!$O$132:$AD$132</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -937,7 +937,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'ADR_Engine'!$O$132:$AD$132</f>
+              <f>'ADR_Engine'!$O$133:$AD$133</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1076,7 +1076,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>133</row>
+      <row>134</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="2880000"/>
@@ -1098,7 +1098,7 @@
     <from>
       <col>13</col>
       <colOff>0</colOff>
-      <row>133</row>
+      <row>134</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="2880000"/>
@@ -5365,7 +5365,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD132"/>
+  <dimension ref="A1:AD133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -11684,418 +11684,461 @@
     <row r="122">
       <c r="A122" s="8" t="inlineStr">
         <is>
-          <t>card v3: last_q residual carry, no lap (card geo)</t>
+          <t>lap-only (K4 residual steps): every 2025-26 residual step laps at its anniversary</t>
         </is>
       </c>
       <c r="C122" s="11" t="n">
-        <v>3.69126637648649</v>
+        <v>2.910732193880174</v>
       </c>
       <c r="D122" s="11" t="n">
-        <v>178.3241057148202</v>
+        <v>176.9871287134339</v>
       </c>
       <c r="E122" s="11" t="n">
-        <v>26.17797871893561</v>
+        <v>25.9817104951321</v>
       </c>
       <c r="F122" s="11" t="n">
-        <v>3.69126637648649</v>
+        <v>1.990747787585442</v>
       </c>
       <c r="G122" s="11" t="n">
-        <v>174.5536872915614</v>
+        <v>171.7051486032933</v>
       </c>
       <c r="H122" s="11" t="n">
-        <v>23.0061759850278</v>
+        <v>22.63073858591405</v>
       </c>
       <c r="I122" s="11" t="n">
-        <v>3.60883637648649</v>
+        <v>0.9435507506529328</v>
       </c>
       <c r="J122" s="11" t="n">
-        <v>192.8726371265034</v>
+        <v>187.8933505203212</v>
       </c>
       <c r="K122" s="11" t="n">
-        <v>32.59933312712161</v>
+        <v>31.75773410494469</v>
       </c>
       <c r="L122" s="11" t="n">
-        <v>3.60883637648649</v>
+        <v>1.013196673597509</v>
       </c>
       <c r="M122" s="11" t="n">
-        <v>189.5761052869207</v>
+        <v>184.8071364608028</v>
       </c>
       <c r="N122" s="11" t="n">
-        <v>29.78240614057524</v>
+        <v>29.03320113799212</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="8" t="inlineStr">
         <is>
-          <t>full lap: ex-NA RNPL sized at the 1H26 residual steps</t>
+          <t>card v3: last_q residual carry, no lap (card geo)</t>
         </is>
       </c>
       <c r="C123" s="11" t="n">
-        <v>3.315947459255554</v>
+        <v>3.69126637648649</v>
       </c>
       <c r="D123" s="11" t="n">
-        <v>177.6812219414954</v>
+        <v>178.3241057148202</v>
       </c>
       <c r="E123" s="11" t="n">
-        <v>26.08360338101152</v>
+        <v>26.17797871893561</v>
       </c>
       <c r="F123" s="11" t="n">
-        <v>2.784074164071932</v>
+        <v>3.69126637648649</v>
       </c>
       <c r="G123" s="11" t="n">
-        <v>173.0340496165458</v>
+        <v>174.5536872915614</v>
       </c>
       <c r="H123" s="11" t="n">
-        <v>22.80588773946074</v>
+        <v>23.0061759850278</v>
       </c>
       <c r="I123" s="11" t="n">
-        <v>1.956877127139422</v>
+        <v>3.60883637648649</v>
       </c>
       <c r="J123" s="11" t="n">
-        <v>189.7864468568733</v>
+        <v>192.8726371265034</v>
       </c>
       <c r="K123" s="11" t="n">
-        <v>32.07770524774872</v>
+        <v>32.59933312712161</v>
       </c>
       <c r="L123" s="11" t="n">
-        <v>1.806523050083998</v>
+        <v>3.60883637648649</v>
       </c>
       <c r="M123" s="11" t="n">
-        <v>186.2647150123214</v>
+        <v>189.5761052869207</v>
       </c>
       <c r="N123" s="11" t="n">
-        <v>29.2621867284357</v>
+        <v>29.78240614057524</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="8" t="inlineStr">
         <is>
-          <t>core mean reversion to the 2023-25 mean</t>
+          <t>full lap: ex-NA RNPL sized at the 1H26 residual steps</t>
         </is>
       </c>
       <c r="C124" s="11" t="n">
-        <v>1.864621082769064</v>
+        <v>3.315947459255554</v>
       </c>
       <c r="D124" s="11" t="n">
-        <v>175.1952449912116</v>
+        <v>177.6812219414954</v>
       </c>
       <c r="E124" s="11" t="n">
-        <v>25.71866196470987</v>
+        <v>26.08360338101152</v>
       </c>
       <c r="F124" s="11" t="n">
-        <v>1.332747787585442</v>
+        <v>2.784074164071932</v>
       </c>
       <c r="G124" s="11" t="n">
-        <v>170.6029328032933</v>
+        <v>173.0340496165458</v>
       </c>
       <c r="H124" s="11" t="n">
-        <v>22.48546654347406</v>
+        <v>22.80588773946074</v>
       </c>
       <c r="I124" s="11" t="n">
-        <v>0.9655507506529332</v>
+        <v>1.956877127139422</v>
       </c>
       <c r="J124" s="11" t="n">
-        <v>187.9344509203212</v>
+        <v>189.7864468568733</v>
       </c>
       <c r="K124" s="11" t="n">
-        <v>31.7646808945527</v>
+        <v>32.07770524774872</v>
       </c>
       <c r="L124" s="11" t="n">
-        <v>1.505196673597509</v>
+        <v>1.806523050083998</v>
       </c>
       <c r="M124" s="11" t="n">
-        <v>185.7110880608028</v>
+        <v>186.2647150123214</v>
       </c>
       <c r="N124" s="11" t="n">
-        <v>29.17521193435212</v>
+        <v>29.2621867284357</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="8" t="inlineStr">
         <is>
-          <t>AR(1) on core (K4 rho 0.747)</t>
+          <t>core mean reversion to the 2023-25 mean</t>
         </is>
       </c>
       <c r="C125" s="11" t="n">
-        <v>3.092067886004471</v>
+        <v>1.864621082769064</v>
       </c>
       <c r="D125" s="11" t="n">
-        <v>177.2977386204736</v>
+        <v>175.1952449912116</v>
       </c>
       <c r="E125" s="11" t="n">
-        <v>26.02730802948552</v>
+        <v>25.71866196470987</v>
       </c>
       <c r="F125" s="11" t="n">
-        <v>2.392956549602292</v>
+        <v>1.332747787585442</v>
       </c>
       <c r="G125" s="11" t="n">
-        <v>172.3788885005477</v>
+        <v>170.6029328032933</v>
       </c>
       <c r="H125" s="11" t="n">
-        <v>22.71953750437219</v>
+        <v>22.48546654347406</v>
       </c>
       <c r="I125" s="11" t="n">
-        <v>1.90083269587952</v>
+        <v>0.9655507506529332</v>
       </c>
       <c r="J125" s="11" t="n">
-        <v>189.6817446503935</v>
+        <v>187.9344509203212</v>
       </c>
       <c r="K125" s="11" t="n">
-        <v>32.06000848080952</v>
+        <v>31.7646808945527</v>
       </c>
       <c r="L125" s="11" t="n">
-        <v>2.347158286681769</v>
+        <v>1.505196673597509</v>
       </c>
       <c r="M125" s="11" t="n">
-        <v>187.2580241325226</v>
+        <v>185.7110880608028</v>
       </c>
       <c r="N125" s="11" t="n">
-        <v>29.41823559121929</v>
+        <v>29.17521193435212</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="8" t="inlineStr">
         <is>
+          <t>AR(1) on core (K4 rho 0.747)</t>
+        </is>
+      </c>
+      <c r="C126" s="11" t="n">
+        <v>3.092067886004471</v>
+      </c>
+      <c r="D126" s="11" t="n">
+        <v>177.2977386204736</v>
+      </c>
+      <c r="E126" s="11" t="n">
+        <v>26.02730802948552</v>
+      </c>
+      <c r="F126" s="11" t="n">
+        <v>2.392956549602292</v>
+      </c>
+      <c r="G126" s="11" t="n">
+        <v>172.3788885005477</v>
+      </c>
+      <c r="H126" s="11" t="n">
+        <v>22.71953750437219</v>
+      </c>
+      <c r="I126" s="11" t="n">
+        <v>1.90083269587952</v>
+      </c>
+      <c r="J126" s="11" t="n">
+        <v>189.6817446503935</v>
+      </c>
+      <c r="K126" s="11" t="n">
+        <v>32.06000848080952</v>
+      </c>
+      <c r="L126" s="11" t="n">
+        <v>2.347158286681769</v>
+      </c>
+      <c r="M126" s="11" t="n">
+        <v>187.2580241325226</v>
+      </c>
+      <c r="N126" s="11" t="n">
+        <v>29.41823559121929</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="8" t="inlineStr">
+        <is>
           <t>base + fee-migration K line (DEC-0008 sensitivity)</t>
         </is>
       </c>
-      <c r="C126" s="11" t="n">
+      <c r="C127" s="11" t="n">
         <v>3.487447459255554</v>
       </c>
-      <c r="D126" s="11" t="n">
+      <c r="D127" s="11" t="n">
         <v>177.9749842914954</v>
       </c>
-      <c r="E126" s="11" t="n">
+      <c r="E127" s="11" t="n">
         <v>26.12672769399152</v>
       </c>
-      <c r="F126" s="11" t="n">
+      <c r="F127" s="11" t="n">
         <v>3.158574164071932</v>
       </c>
-      <c r="G126" s="11" t="n">
+      <c r="G127" s="11" t="n">
         <v>173.6613745665458</v>
       </c>
-      <c r="H126" s="11" t="n">
+      <c r="H127" s="11" t="n">
         <v>22.88856916787073</v>
       </c>
-      <c r="I126" s="11" t="n">
+      <c r="I127" s="11" t="n">
         <v>2.761977127139422</v>
       </c>
-      <c r="J126" s="11" t="n">
+      <c r="J127" s="11" t="n">
         <v>191.2905346768732</v>
       </c>
-      <c r="K126" s="11" t="n">
+      <c r="K127" s="11" t="n">
         <v>32.33192617108512</v>
       </c>
-      <c r="L126" s="11" t="n">
+      <c r="L127" s="11" t="n">
         <v>3.267323050083998</v>
       </c>
-      <c r="M126" s="11" t="n">
+      <c r="M127" s="11" t="n">
         <v>188.9486428523214</v>
       </c>
-      <c r="N126" s="11" t="n">
+      <c r="N127" s="11" t="n">
         <v>29.6838317920997</v>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="8" t="inlineStr">
-        <is>
-          <t>chart helper: ADR $ (printed, then engine)</t>
-        </is>
-      </c>
-      <c r="O129" s="20">
-        <f>O7</f>
-        <v/>
-      </c>
-      <c r="P129" s="20">
-        <f>P7</f>
-        <v/>
-      </c>
-      <c r="Q129" s="20">
-        <f>Q7</f>
-        <v/>
-      </c>
-      <c r="R129" s="20">
-        <f>R7</f>
-        <v/>
-      </c>
-      <c r="S129" s="20">
-        <f>S7</f>
-        <v/>
-      </c>
-      <c r="T129" s="20">
-        <f>T7</f>
-        <v/>
-      </c>
-      <c r="U129" s="20">
-        <f>U7</f>
-        <v/>
-      </c>
-      <c r="V129" s="20">
-        <f>V7</f>
-        <v/>
-      </c>
-      <c r="W129" s="20">
-        <f>W7</f>
-        <v/>
-      </c>
-      <c r="X129" s="20">
-        <f>X7</f>
-        <v/>
-      </c>
-      <c r="Y129" s="20">
-        <f>Y7</f>
-        <v/>
-      </c>
-      <c r="Z129" s="20">
-        <f>Z7</f>
-        <v/>
-      </c>
-      <c r="AA129" s="20">
-        <f>AA7</f>
-        <v/>
-      </c>
-      <c r="AB129" s="20">
-        <f>AB7</f>
-        <v/>
-      </c>
-      <c r="AC129" s="20">
-        <f>AC7</f>
-        <v/>
-      </c>
-      <c r="AD129" s="20">
-        <f>AD7</f>
-        <v/>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="8" t="inlineStr">
         <is>
-          <t>chart helper: Street ADR $</t>
-        </is>
+          <t>chart helper: ADR $ (printed, then engine)</t>
+        </is>
+      </c>
+      <c r="O130" s="20">
+        <f>O7</f>
+        <v/>
+      </c>
+      <c r="P130" s="20">
+        <f>P7</f>
+        <v/>
+      </c>
+      <c r="Q130" s="20">
+        <f>Q7</f>
+        <v/>
+      </c>
+      <c r="R130" s="20">
+        <f>R7</f>
+        <v/>
+      </c>
+      <c r="S130" s="20">
+        <f>S7</f>
+        <v/>
+      </c>
+      <c r="T130" s="20">
+        <f>T7</f>
+        <v/>
+      </c>
+      <c r="U130" s="20">
+        <f>U7</f>
+        <v/>
+      </c>
+      <c r="V130" s="20">
+        <f>V7</f>
+        <v/>
+      </c>
+      <c r="W130" s="20">
+        <f>W7</f>
+        <v/>
+      </c>
+      <c r="X130" s="20">
+        <f>X7</f>
+        <v/>
       </c>
       <c r="Y130" s="20">
-        <f>Y100</f>
+        <f>Y7</f>
         <v/>
       </c>
       <c r="Z130" s="20">
-        <f>Z100</f>
+        <f>Z7</f>
+        <v/>
+      </c>
+      <c r="AA130" s="20">
+        <f>AA7</f>
+        <v/>
+      </c>
+      <c r="AB130" s="20">
+        <f>AB7</f>
+        <v/>
+      </c>
+      <c r="AC130" s="20">
+        <f>AC7</f>
+        <v/>
+      </c>
+      <c r="AD130" s="20">
+        <f>AD7</f>
         <v/>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="8" t="inlineStr">
         <is>
-          <t>chart helper: FX identity (pp)</t>
-        </is>
-      </c>
-      <c r="O131" s="20">
-        <f>O51</f>
-        <v/>
-      </c>
-      <c r="P131" s="20">
-        <f>P51</f>
-        <v/>
-      </c>
-      <c r="Q131" s="20">
-        <f>Q51</f>
-        <v/>
-      </c>
-      <c r="R131" s="20">
-        <f>R51</f>
-        <v/>
-      </c>
-      <c r="S131" s="20">
-        <f>S51</f>
-        <v/>
-      </c>
-      <c r="T131" s="20">
-        <f>T51</f>
-        <v/>
-      </c>
-      <c r="U131" s="20">
-        <f>U51</f>
-        <v/>
-      </c>
-      <c r="V131" s="20">
-        <f>V51</f>
-        <v/>
-      </c>
-      <c r="W131" s="20">
-        <f>W51</f>
-        <v/>
-      </c>
-      <c r="X131" s="20">
-        <f>X51</f>
-        <v/>
+          <t>chart helper: Street ADR $</t>
+        </is>
       </c>
       <c r="Y131" s="20">
-        <f>Y51</f>
+        <f>Y100</f>
         <v/>
       </c>
       <c r="Z131" s="20">
-        <f>Z51</f>
-        <v/>
-      </c>
-      <c r="AA131" s="20">
-        <f>AA51</f>
-        <v/>
-      </c>
-      <c r="AB131" s="20">
-        <f>AB51</f>
-        <v/>
-      </c>
-      <c r="AC131" s="20">
-        <f>AC51</f>
-        <v/>
-      </c>
-      <c r="AD131" s="20">
-        <f>AD51</f>
+        <f>Z100</f>
         <v/>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="8" t="inlineStr">
         <is>
+          <t>chart helper: FX identity (pp)</t>
+        </is>
+      </c>
+      <c r="O132" s="20">
+        <f>O51</f>
+        <v/>
+      </c>
+      <c r="P132" s="20">
+        <f>P51</f>
+        <v/>
+      </c>
+      <c r="Q132" s="20">
+        <f>Q51</f>
+        <v/>
+      </c>
+      <c r="R132" s="20">
+        <f>R51</f>
+        <v/>
+      </c>
+      <c r="S132" s="20">
+        <f>S51</f>
+        <v/>
+      </c>
+      <c r="T132" s="20">
+        <f>T51</f>
+        <v/>
+      </c>
+      <c r="U132" s="20">
+        <f>U51</f>
+        <v/>
+      </c>
+      <c r="V132" s="20">
+        <f>V51</f>
+        <v/>
+      </c>
+      <c r="W132" s="20">
+        <f>W51</f>
+        <v/>
+      </c>
+      <c r="X132" s="20">
+        <f>X51</f>
+        <v/>
+      </c>
+      <c r="Y132" s="20">
+        <f>Y51</f>
+        <v/>
+      </c>
+      <c r="Z132" s="20">
+        <f>Z51</f>
+        <v/>
+      </c>
+      <c r="AA132" s="20">
+        <f>AA51</f>
+        <v/>
+      </c>
+      <c r="AB132" s="20">
+        <f>AB51</f>
+        <v/>
+      </c>
+      <c r="AC132" s="20">
+        <f>AC51</f>
+        <v/>
+      </c>
+      <c r="AD132" s="20">
+        <f>AD51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="8" t="inlineStr">
+        <is>
           <t>chart helper: disclosed FX (pp)</t>
         </is>
       </c>
-      <c r="O132" s="20">
+      <c r="O133" s="20">
         <f>O10</f>
         <v/>
       </c>
-      <c r="P132" s="20">
+      <c r="P133" s="20">
         <f>P10</f>
         <v/>
       </c>
-      <c r="Q132" s="20">
+      <c r="Q133" s="20">
         <f>Q10</f>
         <v/>
       </c>
-      <c r="R132" s="20">
+      <c r="R133" s="20">
         <f>R10</f>
         <v/>
       </c>
-      <c r="S132" s="20">
+      <c r="S133" s="20">
         <f>S10</f>
         <v/>
       </c>
-      <c r="T132" s="20">
+      <c r="T133" s="20">
         <f>T10</f>
         <v/>
       </c>
-      <c r="U132" s="20">
+      <c r="U133" s="20">
         <f>U10</f>
         <v/>
       </c>
-      <c r="V132" s="20">
+      <c r="V133" s="20">
         <f>V10</f>
         <v/>
       </c>
-      <c r="W132" s="20">
+      <c r="W133" s="20">
         <f>W10</f>
         <v/>
       </c>
-      <c r="X132" s="20">
+      <c r="X133" s="20">
         <f>X10</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
ADR line v2: sub-regional (country-level) geographic mix from the 123-market panel and June-2026 listed prices in USD (30 countries), pre-registered; H1 attribution -0.45pp 2023-26 fading to -0.15 (EMEA +0.4 in 2Q26), H2 fails, H3 forward -0.13 to -0.18pp; four-region composition tilt sensitivity (LatAm 30 / APAC 25 / EMEA 5 -> -1.70pp) and the share-shift lever; scenarios in the alternatives and workbook
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model/ABNB_official_model.xlsx
+++ b/model/ABNB_official_model.xlsx
@@ -787,7 +787,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'ADR_Engine'!$O$130:$AD$130</f>
+              <f>'ADR_Engine'!$O$132:$AD$132</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -818,7 +818,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'ADR_Engine'!$O$131:$AD$131</f>
+              <f>'ADR_Engine'!$O$133:$AD$133</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -906,7 +906,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'ADR_Engine'!$O$132:$AD$132</f>
+              <f>'ADR_Engine'!$O$134:$AD$134</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -937,7 +937,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'ADR_Engine'!$O$133:$AD$133</f>
+              <f>'ADR_Engine'!$O$135:$AD$135</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1076,7 +1076,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>134</row>
+      <row>136</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="2880000"/>
@@ -1098,7 +1098,7 @@
     <from>
       <col>13</col>
       <colOff>0</colOff>
-      <row>134</row>
+      <row>136</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="2880000"/>
@@ -5365,7 +5365,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD133"/>
+  <dimension ref="A1:AD135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -11684,461 +11684,547 @@
     <row r="122">
       <c r="A122" s="8" t="inlineStr">
         <is>
-          <t>lap-only (K4 residual steps): every 2025-26 residual step laps at its anniversary</t>
+          <t>base + sub-regional country mix (v2 H3, Inside Airbnb panel)</t>
         </is>
       </c>
       <c r="C122" s="11" t="n">
-        <v>2.910732193880174</v>
+        <v>3.182081964103476</v>
       </c>
       <c r="D122" s="11" t="n">
-        <v>176.9871287134339</v>
+        <v>177.4519237348494</v>
       </c>
       <c r="E122" s="11" t="n">
-        <v>25.9817104951321</v>
+        <v>26.04994240427589</v>
       </c>
       <c r="F122" s="11" t="n">
-        <v>1.990747787585442</v>
+        <v>2.640676678321757</v>
       </c>
       <c r="G122" s="11" t="n">
-        <v>171.7051486032933</v>
+        <v>172.7938444881657</v>
       </c>
       <c r="H122" s="11" t="n">
-        <v>22.63073858591405</v>
+        <v>22.77422870354024</v>
       </c>
       <c r="I122" s="11" t="n">
-        <v>0.9435507506529328</v>
+        <v>2.265309708688182</v>
       </c>
       <c r="J122" s="11" t="n">
-        <v>187.8933505203212</v>
+        <v>190.3626606057227</v>
       </c>
       <c r="K122" s="11" t="n">
-        <v>31.75773410494469</v>
+        <v>32.17509689557925</v>
       </c>
       <c r="L122" s="11" t="n">
-        <v>1.013196673597509</v>
+        <v>2.795333000538972</v>
       </c>
       <c r="M122" s="11" t="n">
-        <v>184.8071364608028</v>
+        <v>188.0814555342924</v>
       </c>
       <c r="N122" s="11" t="n">
-        <v>29.03320113799212</v>
+        <v>29.54759666443733</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="8" t="inlineStr">
         <is>
-          <t>card v3: last_q residual carry, no lap (card geo)</t>
+          <t>base + sub-regional + composition tilt B (EMEA 5 / LatAm 30 / APAC 25)</t>
         </is>
       </c>
       <c r="C123" s="11" t="n">
-        <v>3.69126637648649</v>
+        <v>2.800767198387953</v>
       </c>
       <c r="D123" s="11" t="n">
-        <v>178.3241057148202</v>
+        <v>176.7987696726552</v>
       </c>
       <c r="E123" s="11" t="n">
-        <v>26.17797871893561</v>
+        <v>25.95405938794579</v>
       </c>
       <c r="F123" s="11" t="n">
-        <v>3.69126637648649</v>
+        <v>2.276405895791162</v>
       </c>
       <c r="G123" s="11" t="n">
-        <v>174.5536872915614</v>
+        <v>172.1836545003487</v>
       </c>
       <c r="H123" s="11" t="n">
-        <v>23.0061759850278</v>
+        <v>22.69380566314596</v>
       </c>
       <c r="I123" s="11" t="n">
-        <v>3.60883637648649</v>
+        <v>1.845411024644575</v>
       </c>
       <c r="J123" s="11" t="n">
-        <v>192.8726371265034</v>
+        <v>189.5782058841924</v>
       </c>
       <c r="K123" s="11" t="n">
-        <v>32.59933312712161</v>
+        <v>32.0425083585462</v>
       </c>
       <c r="L123" s="11" t="n">
-        <v>3.60883637648649</v>
+        <v>2.514402127934693</v>
       </c>
       <c r="M123" s="11" t="n">
-        <v>189.5761052869207</v>
+        <v>187.5653012420565</v>
       </c>
       <c r="N123" s="11" t="n">
-        <v>29.78240614057524</v>
+        <v>29.46650882512708</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="8" t="inlineStr">
         <is>
-          <t>full lap: ex-NA RNPL sized at the 1H26 residual steps</t>
+          <t>lap-only (K4 residual steps): every 2025-26 residual step laps at its anniversary</t>
         </is>
       </c>
       <c r="C124" s="11" t="n">
-        <v>3.315947459255554</v>
+        <v>2.910732193880174</v>
       </c>
       <c r="D124" s="11" t="n">
-        <v>177.6812219414954</v>
+        <v>176.9871287134339</v>
       </c>
       <c r="E124" s="11" t="n">
-        <v>26.08360338101152</v>
+        <v>25.9817104951321</v>
       </c>
       <c r="F124" s="11" t="n">
-        <v>2.784074164071932</v>
+        <v>1.990747787585442</v>
       </c>
       <c r="G124" s="11" t="n">
-        <v>173.0340496165458</v>
+        <v>171.7051486032933</v>
       </c>
       <c r="H124" s="11" t="n">
-        <v>22.80588773946074</v>
+        <v>22.63073858591405</v>
       </c>
       <c r="I124" s="11" t="n">
-        <v>1.956877127139422</v>
+        <v>0.9435507506529328</v>
       </c>
       <c r="J124" s="11" t="n">
-        <v>189.7864468568733</v>
+        <v>187.8933505203212</v>
       </c>
       <c r="K124" s="11" t="n">
-        <v>32.07770524774872</v>
+        <v>31.75773410494469</v>
       </c>
       <c r="L124" s="11" t="n">
-        <v>1.806523050083998</v>
+        <v>1.013196673597509</v>
       </c>
       <c r="M124" s="11" t="n">
-        <v>186.2647150123214</v>
+        <v>184.8071364608028</v>
       </c>
       <c r="N124" s="11" t="n">
-        <v>29.2621867284357</v>
+        <v>29.03320113799212</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="8" t="inlineStr">
         <is>
-          <t>core mean reversion to the 2023-25 mean</t>
+          <t>card v3: last_q residual carry, no lap (card geo)</t>
         </is>
       </c>
       <c r="C125" s="11" t="n">
-        <v>1.864621082769064</v>
+        <v>3.69126637648649</v>
       </c>
       <c r="D125" s="11" t="n">
-        <v>175.1952449912116</v>
+        <v>178.3241057148202</v>
       </c>
       <c r="E125" s="11" t="n">
-        <v>25.71866196470987</v>
+        <v>26.17797871893561</v>
       </c>
       <c r="F125" s="11" t="n">
-        <v>1.332747787585442</v>
+        <v>3.69126637648649</v>
       </c>
       <c r="G125" s="11" t="n">
-        <v>170.6029328032933</v>
+        <v>174.5536872915614</v>
       </c>
       <c r="H125" s="11" t="n">
-        <v>22.48546654347406</v>
+        <v>23.0061759850278</v>
       </c>
       <c r="I125" s="11" t="n">
-        <v>0.9655507506529332</v>
+        <v>3.60883637648649</v>
       </c>
       <c r="J125" s="11" t="n">
-        <v>187.9344509203212</v>
+        <v>192.8726371265034</v>
       </c>
       <c r="K125" s="11" t="n">
-        <v>31.7646808945527</v>
+        <v>32.59933312712161</v>
       </c>
       <c r="L125" s="11" t="n">
-        <v>1.505196673597509</v>
+        <v>3.60883637648649</v>
       </c>
       <c r="M125" s="11" t="n">
-        <v>185.7110880608028</v>
+        <v>189.5761052869207</v>
       </c>
       <c r="N125" s="11" t="n">
-        <v>29.17521193435212</v>
+        <v>29.78240614057524</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="8" t="inlineStr">
         <is>
-          <t>AR(1) on core (K4 rho 0.747)</t>
+          <t>full lap: ex-NA RNPL sized at the 1H26 residual steps</t>
         </is>
       </c>
       <c r="C126" s="11" t="n">
-        <v>3.092067886004471</v>
+        <v>3.315947459255554</v>
       </c>
       <c r="D126" s="11" t="n">
-        <v>177.2977386204736</v>
+        <v>177.6812219414954</v>
       </c>
       <c r="E126" s="11" t="n">
-        <v>26.02730802948552</v>
+        <v>26.08360338101152</v>
       </c>
       <c r="F126" s="11" t="n">
-        <v>2.392956549602292</v>
+        <v>2.784074164071932</v>
       </c>
       <c r="G126" s="11" t="n">
-        <v>172.3788885005477</v>
+        <v>173.0340496165458</v>
       </c>
       <c r="H126" s="11" t="n">
-        <v>22.71953750437219</v>
+        <v>22.80588773946074</v>
       </c>
       <c r="I126" s="11" t="n">
-        <v>1.90083269587952</v>
+        <v>1.956877127139422</v>
       </c>
       <c r="J126" s="11" t="n">
-        <v>189.6817446503935</v>
+        <v>189.7864468568733</v>
       </c>
       <c r="K126" s="11" t="n">
-        <v>32.06000848080952</v>
+        <v>32.07770524774872</v>
       </c>
       <c r="L126" s="11" t="n">
-        <v>2.347158286681769</v>
+        <v>1.806523050083998</v>
       </c>
       <c r="M126" s="11" t="n">
-        <v>187.2580241325226</v>
+        <v>186.2647150123214</v>
       </c>
       <c r="N126" s="11" t="n">
-        <v>29.41823559121929</v>
+        <v>29.2621867284357</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="8" t="inlineStr">
         <is>
+          <t>core mean reversion to the 2023-25 mean</t>
+        </is>
+      </c>
+      <c r="C127" s="11" t="n">
+        <v>1.864621082769064</v>
+      </c>
+      <c r="D127" s="11" t="n">
+        <v>175.1952449912116</v>
+      </c>
+      <c r="E127" s="11" t="n">
+        <v>25.71866196470987</v>
+      </c>
+      <c r="F127" s="11" t="n">
+        <v>1.332747787585442</v>
+      </c>
+      <c r="G127" s="11" t="n">
+        <v>170.6029328032933</v>
+      </c>
+      <c r="H127" s="11" t="n">
+        <v>22.48546654347406</v>
+      </c>
+      <c r="I127" s="11" t="n">
+        <v>0.9655507506529332</v>
+      </c>
+      <c r="J127" s="11" t="n">
+        <v>187.9344509203212</v>
+      </c>
+      <c r="K127" s="11" t="n">
+        <v>31.7646808945527</v>
+      </c>
+      <c r="L127" s="11" t="n">
+        <v>1.505196673597509</v>
+      </c>
+      <c r="M127" s="11" t="n">
+        <v>185.7110880608028</v>
+      </c>
+      <c r="N127" s="11" t="n">
+        <v>29.17521193435212</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="8" t="inlineStr">
+        <is>
+          <t>AR(1) on core (K4 rho 0.747)</t>
+        </is>
+      </c>
+      <c r="C128" s="11" t="n">
+        <v>3.092067886004471</v>
+      </c>
+      <c r="D128" s="11" t="n">
+        <v>177.2977386204736</v>
+      </c>
+      <c r="E128" s="11" t="n">
+        <v>26.02730802948552</v>
+      </c>
+      <c r="F128" s="11" t="n">
+        <v>2.392956549602292</v>
+      </c>
+      <c r="G128" s="11" t="n">
+        <v>172.3788885005477</v>
+      </c>
+      <c r="H128" s="11" t="n">
+        <v>22.71953750437219</v>
+      </c>
+      <c r="I128" s="11" t="n">
+        <v>1.90083269587952</v>
+      </c>
+      <c r="J128" s="11" t="n">
+        <v>189.6817446503935</v>
+      </c>
+      <c r="K128" s="11" t="n">
+        <v>32.06000848080952</v>
+      </c>
+      <c r="L128" s="11" t="n">
+        <v>2.347158286681769</v>
+      </c>
+      <c r="M128" s="11" t="n">
+        <v>187.2580241325226</v>
+      </c>
+      <c r="N128" s="11" t="n">
+        <v>29.41823559121929</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="8" t="inlineStr">
+        <is>
           <t>base + fee-migration K line (DEC-0008 sensitivity)</t>
         </is>
       </c>
-      <c r="C127" s="11" t="n">
+      <c r="C129" s="11" t="n">
         <v>3.487447459255554</v>
       </c>
-      <c r="D127" s="11" t="n">
+      <c r="D129" s="11" t="n">
         <v>177.9749842914954</v>
       </c>
-      <c r="E127" s="11" t="n">
+      <c r="E129" s="11" t="n">
         <v>26.12672769399152</v>
       </c>
-      <c r="F127" s="11" t="n">
+      <c r="F129" s="11" t="n">
         <v>3.158574164071932</v>
       </c>
-      <c r="G127" s="11" t="n">
+      <c r="G129" s="11" t="n">
         <v>173.6613745665458</v>
       </c>
-      <c r="H127" s="11" t="n">
+      <c r="H129" s="11" t="n">
         <v>22.88856916787073</v>
       </c>
-      <c r="I127" s="11" t="n">
+      <c r="I129" s="11" t="n">
         <v>2.761977127139422</v>
       </c>
-      <c r="J127" s="11" t="n">
+      <c r="J129" s="11" t="n">
         <v>191.2905346768732</v>
       </c>
-      <c r="K127" s="11" t="n">
+      <c r="K129" s="11" t="n">
         <v>32.33192617108512</v>
       </c>
-      <c r="L127" s="11" t="n">
+      <c r="L129" s="11" t="n">
         <v>3.267323050083998</v>
       </c>
-      <c r="M127" s="11" t="n">
+      <c r="M129" s="11" t="n">
         <v>188.9486428523214</v>
       </c>
-      <c r="N127" s="11" t="n">
+      <c r="N129" s="11" t="n">
         <v>29.6838317920997</v>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="8" t="inlineStr">
-        <is>
-          <t>chart helper: ADR $ (printed, then engine)</t>
-        </is>
-      </c>
-      <c r="O130" s="20">
-        <f>O7</f>
-        <v/>
-      </c>
-      <c r="P130" s="20">
-        <f>P7</f>
-        <v/>
-      </c>
-      <c r="Q130" s="20">
-        <f>Q7</f>
-        <v/>
-      </c>
-      <c r="R130" s="20">
-        <f>R7</f>
-        <v/>
-      </c>
-      <c r="S130" s="20">
-        <f>S7</f>
-        <v/>
-      </c>
-      <c r="T130" s="20">
-        <f>T7</f>
-        <v/>
-      </c>
-      <c r="U130" s="20">
-        <f>U7</f>
-        <v/>
-      </c>
-      <c r="V130" s="20">
-        <f>V7</f>
-        <v/>
-      </c>
-      <c r="W130" s="20">
-        <f>W7</f>
-        <v/>
-      </c>
-      <c r="X130" s="20">
-        <f>X7</f>
-        <v/>
-      </c>
-      <c r="Y130" s="20">
-        <f>Y7</f>
-        <v/>
-      </c>
-      <c r="Z130" s="20">
-        <f>Z7</f>
-        <v/>
-      </c>
-      <c r="AA130" s="20">
-        <f>AA7</f>
-        <v/>
-      </c>
-      <c r="AB130" s="20">
-        <f>AB7</f>
-        <v/>
-      </c>
-      <c r="AC130" s="20">
-        <f>AC7</f>
-        <v/>
-      </c>
-      <c r="AD130" s="20">
-        <f>AD7</f>
-        <v/>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="8" t="inlineStr">
-        <is>
-          <t>chart helper: Street ADR $</t>
-        </is>
-      </c>
-      <c r="Y131" s="20">
-        <f>Y100</f>
-        <v/>
-      </c>
-      <c r="Z131" s="20">
-        <f>Z100</f>
-        <v/>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="8" t="inlineStr">
         <is>
-          <t>chart helper: FX identity (pp)</t>
+          <t>chart helper: ADR $ (printed, then engine)</t>
         </is>
       </c>
       <c r="O132" s="20">
-        <f>O51</f>
+        <f>O7</f>
         <v/>
       </c>
       <c r="P132" s="20">
-        <f>P51</f>
+        <f>P7</f>
         <v/>
       </c>
       <c r="Q132" s="20">
-        <f>Q51</f>
+        <f>Q7</f>
         <v/>
       </c>
       <c r="R132" s="20">
-        <f>R51</f>
+        <f>R7</f>
         <v/>
       </c>
       <c r="S132" s="20">
-        <f>S51</f>
+        <f>S7</f>
         <v/>
       </c>
       <c r="T132" s="20">
-        <f>T51</f>
+        <f>T7</f>
         <v/>
       </c>
       <c r="U132" s="20">
-        <f>U51</f>
+        <f>U7</f>
         <v/>
       </c>
       <c r="V132" s="20">
-        <f>V51</f>
+        <f>V7</f>
         <v/>
       </c>
       <c r="W132" s="20">
-        <f>W51</f>
+        <f>W7</f>
         <v/>
       </c>
       <c r="X132" s="20">
-        <f>X51</f>
+        <f>X7</f>
         <v/>
       </c>
       <c r="Y132" s="20">
-        <f>Y51</f>
+        <f>Y7</f>
         <v/>
       </c>
       <c r="Z132" s="20">
-        <f>Z51</f>
+        <f>Z7</f>
         <v/>
       </c>
       <c r="AA132" s="20">
-        <f>AA51</f>
+        <f>AA7</f>
         <v/>
       </c>
       <c r="AB132" s="20">
-        <f>AB51</f>
+        <f>AB7</f>
         <v/>
       </c>
       <c r="AC132" s="20">
-        <f>AC51</f>
+        <f>AC7</f>
         <v/>
       </c>
       <c r="AD132" s="20">
-        <f>AD51</f>
+        <f>AD7</f>
         <v/>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="8" t="inlineStr">
         <is>
+          <t>chart helper: Street ADR $</t>
+        </is>
+      </c>
+      <c r="Y133" s="20">
+        <f>Y100</f>
+        <v/>
+      </c>
+      <c r="Z133" s="20">
+        <f>Z100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="8" t="inlineStr">
+        <is>
+          <t>chart helper: FX identity (pp)</t>
+        </is>
+      </c>
+      <c r="O134" s="20">
+        <f>O51</f>
+        <v/>
+      </c>
+      <c r="P134" s="20">
+        <f>P51</f>
+        <v/>
+      </c>
+      <c r="Q134" s="20">
+        <f>Q51</f>
+        <v/>
+      </c>
+      <c r="R134" s="20">
+        <f>R51</f>
+        <v/>
+      </c>
+      <c r="S134" s="20">
+        <f>S51</f>
+        <v/>
+      </c>
+      <c r="T134" s="20">
+        <f>T51</f>
+        <v/>
+      </c>
+      <c r="U134" s="20">
+        <f>U51</f>
+        <v/>
+      </c>
+      <c r="V134" s="20">
+        <f>V51</f>
+        <v/>
+      </c>
+      <c r="W134" s="20">
+        <f>W51</f>
+        <v/>
+      </c>
+      <c r="X134" s="20">
+        <f>X51</f>
+        <v/>
+      </c>
+      <c r="Y134" s="20">
+        <f>Y51</f>
+        <v/>
+      </c>
+      <c r="Z134" s="20">
+        <f>Z51</f>
+        <v/>
+      </c>
+      <c r="AA134" s="20">
+        <f>AA51</f>
+        <v/>
+      </c>
+      <c r="AB134" s="20">
+        <f>AB51</f>
+        <v/>
+      </c>
+      <c r="AC134" s="20">
+        <f>AC51</f>
+        <v/>
+      </c>
+      <c r="AD134" s="20">
+        <f>AD51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="8" t="inlineStr">
+        <is>
           <t>chart helper: disclosed FX (pp)</t>
         </is>
       </c>
-      <c r="O133" s="20">
+      <c r="O135" s="20">
         <f>O10</f>
         <v/>
       </c>
-      <c r="P133" s="20">
+      <c r="P135" s="20">
         <f>P10</f>
         <v/>
       </c>
-      <c r="Q133" s="20">
+      <c r="Q135" s="20">
         <f>Q10</f>
         <v/>
       </c>
-      <c r="R133" s="20">
+      <c r="R135" s="20">
         <f>R10</f>
         <v/>
       </c>
-      <c r="S133" s="20">
+      <c r="S135" s="20">
         <f>S10</f>
         <v/>
       </c>
-      <c r="T133" s="20">
+      <c r="T135" s="20">
         <f>T10</f>
         <v/>
       </c>
-      <c r="U133" s="20">
+      <c r="U135" s="20">
         <f>U10</f>
         <v/>
       </c>
-      <c r="V133" s="20">
+      <c r="V135" s="20">
         <f>V10</f>
         <v/>
       </c>
-      <c r="W133" s="20">
+      <c r="W135" s="20">
         <f>W10</f>
         <v/>
       </c>
-      <c r="X133" s="20">
+      <c r="X135" s="20">
         <f>X10</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
ADR line v2: Hong Kong priced in HKD (was CNY); sub-regional term rebuilt (means unchanged: -0.45pp 2023-26, -0.15 last four quarters, forward -0.14 to -0.18); origin-destination inventory archived; reviewer-language origin exhibit (English 71% -> 58% of panel reviews 2022-26, Spanish 11 -> 16, Portuguese 1.8 -> 3.5), figure adr_origin_language_shares; no price link, descriptive only
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model/ABNB_official_model.xlsx
+++ b/model/ABNB_official_model.xlsx
@@ -11688,40 +11688,40 @@
         </is>
       </c>
       <c r="C122" s="11" t="n">
-        <v>3.182081964103476</v>
+        <v>3.178728196637815</v>
       </c>
       <c r="D122" s="11" t="n">
-        <v>177.4519237348494</v>
+        <v>177.4461790665574</v>
       </c>
       <c r="E122" s="11" t="n">
-        <v>26.04994240427589</v>
+        <v>26.04909908697064</v>
       </c>
       <c r="F122" s="11" t="n">
-        <v>2.640676678321757</v>
+        <v>2.637266387956136</v>
       </c>
       <c r="G122" s="11" t="n">
-        <v>172.7938444881657</v>
+        <v>172.7881319107742</v>
       </c>
       <c r="H122" s="11" t="n">
-        <v>22.77422870354024</v>
+        <v>22.77347578584005</v>
       </c>
       <c r="I122" s="11" t="n">
-        <v>2.265309708688182</v>
+        <v>2.261923490219556</v>
       </c>
       <c r="J122" s="11" t="n">
-        <v>190.3626606057227</v>
+        <v>190.3563344723796</v>
       </c>
       <c r="K122" s="11" t="n">
-        <v>32.17509689557925</v>
+        <v>32.1740276525216</v>
       </c>
       <c r="L122" s="11" t="n">
-        <v>2.795333000538972</v>
+        <v>2.79184921359367</v>
       </c>
       <c r="M122" s="11" t="n">
-        <v>188.0814555342924</v>
+        <v>188.0750547725378</v>
       </c>
       <c r="N122" s="11" t="n">
-        <v>29.54759666443733</v>
+        <v>29.54659110476569</v>
       </c>
     </row>
     <row r="123">
@@ -11731,40 +11731,40 @@
         </is>
       </c>
       <c r="C123" s="11" t="n">
-        <v>2.800767198387953</v>
+        <v>2.797413430922292</v>
       </c>
       <c r="D123" s="11" t="n">
-        <v>176.7987696726552</v>
+        <v>176.7930250043633</v>
       </c>
       <c r="E123" s="11" t="n">
-        <v>25.95405938794579</v>
+        <v>25.95321607064054</v>
       </c>
       <c r="F123" s="11" t="n">
-        <v>2.276405895791162</v>
+        <v>2.27299560542554</v>
       </c>
       <c r="G123" s="11" t="n">
-        <v>172.1836545003487</v>
+        <v>172.1779419229572</v>
       </c>
       <c r="H123" s="11" t="n">
-        <v>22.69380566314596</v>
+        <v>22.69305274544576</v>
       </c>
       <c r="I123" s="11" t="n">
-        <v>1.845411024644575</v>
+        <v>1.842024806175949</v>
       </c>
       <c r="J123" s="11" t="n">
-        <v>189.5782058841924</v>
+        <v>189.5718797508493</v>
       </c>
       <c r="K123" s="11" t="n">
-        <v>32.0425083585462</v>
+        <v>32.04143911548855</v>
       </c>
       <c r="L123" s="11" t="n">
-        <v>2.514402127934693</v>
+        <v>2.510918340989391</v>
       </c>
       <c r="M123" s="11" t="n">
-        <v>187.5653012420565</v>
+        <v>187.5589004803019</v>
       </c>
       <c r="N123" s="11" t="n">
-        <v>29.46650882512708</v>
+        <v>29.46550326545543</v>
       </c>
     </row>
     <row r="124">

</xml_diff>

<commit_message>
ADR line v2 upgrades 1/2/3/6: Eurostat reweight of the EMEA mix (weights move, term moves 0.02pp), origin-to-destination layer from tourism boards (implied ex-NA split 10.5/16.4/14.9, tilt B retired, ordering p 0.018), reconciliation to the 10-K (four-region term within 0.02-0.09pp for 2023-25; EMEA slope 1.09 vs identity 1.0, n 7) and to the EMEA disclosures, refresh_prices + geomix stage in run.py + 17 new tests (27 total) + eight pre-registered score lines; six-panel figure adr_geomix_logic; ten-sentence thesis adr_v2_thesis.md; DEC-0037/38/39 proposed
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/model/ABNB_official_model.xlsx
+++ b/model/ABNB_official_model.xlsx
@@ -787,7 +787,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'ADR_Engine'!$O$132:$AD$132</f>
+              <f>'ADR_Engine'!$O$133:$AD$133</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -818,7 +818,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'ADR_Engine'!$O$133:$AD$133</f>
+              <f>'ADR_Engine'!$O$134:$AD$134</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -906,7 +906,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'ADR_Engine'!$O$134:$AD$134</f>
+              <f>'ADR_Engine'!$O$135:$AD$135</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -937,7 +937,7 @@
           </cat>
           <val>
             <numRef>
-              <f>'ADR_Engine'!$O$135:$AD$135</f>
+              <f>'ADR_Engine'!$O$136:$AD$136</f>
             </numRef>
           </val>
           <smooth val="0"/>
@@ -1076,7 +1076,7 @@
     <from>
       <col>2</col>
       <colOff>0</colOff>
-      <row>136</row>
+      <row>137</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="2880000"/>
@@ -1098,7 +1098,7 @@
     <from>
       <col>13</col>
       <colOff>0</colOff>
-      <row>136</row>
+      <row>137</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="7920000" cy="2880000"/>
@@ -5365,7 +5365,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AD135"/>
+  <dimension ref="A1:AD136"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -11706,7 +11706,7 @@
         <v>22.77347578584005</v>
       </c>
       <c r="I122" s="11" t="n">
-        <v>2.261923490219556</v>
+        <v>2.261923490219557</v>
       </c>
       <c r="J122" s="11" t="n">
         <v>190.3563344723796</v>
@@ -11715,7 +11715,7 @@
         <v>32.1740276525216</v>
       </c>
       <c r="L122" s="11" t="n">
-        <v>2.79184921359367</v>
+        <v>2.791849213593684</v>
       </c>
       <c r="M122" s="11" t="n">
         <v>188.0750547725378</v>
@@ -11727,504 +11727,547 @@
     <row r="123">
       <c r="A123" s="8" t="inlineStr">
         <is>
-          <t>base + sub-regional + composition tilt B (EMEA 5 / LatAm 30 / APAC 25)</t>
+          <t>base + sub-regional + measured origin-destination tilt (upgrade 2: EMEA 10.5 / LatAm 16.4 / APAC 14.9)</t>
         </is>
       </c>
       <c r="C123" s="11" t="n">
-        <v>2.797413430922292</v>
+        <v>3.441974423799111</v>
       </c>
       <c r="D123" s="11" t="n">
-        <v>176.7930250043633</v>
+        <v>177.897093529062</v>
       </c>
       <c r="E123" s="11" t="n">
-        <v>25.95321607064054</v>
+        <v>26.11529333006631</v>
       </c>
       <c r="F123" s="11" t="n">
-        <v>2.27299560542554</v>
+        <v>2.878353163829614</v>
       </c>
       <c r="G123" s="11" t="n">
-        <v>172.1779419229572</v>
+        <v>173.1919763690399</v>
       </c>
       <c r="H123" s="11" t="n">
-        <v>22.69305274544576</v>
+        <v>22.82670248543946</v>
       </c>
       <c r="I123" s="11" t="n">
-        <v>1.842024806175949</v>
+        <v>2.547238721983384</v>
       </c>
       <c r="J123" s="11" t="n">
-        <v>189.5718797508493</v>
+        <v>190.8893603883608</v>
       </c>
       <c r="K123" s="11" t="n">
-        <v>32.04143911548855</v>
+        <v>32.26411969284074</v>
       </c>
       <c r="L123" s="11" t="n">
-        <v>2.510918340989391</v>
+        <v>2.977560195437551</v>
       </c>
       <c r="M123" s="11" t="n">
-        <v>187.5589004803019</v>
+        <v>188.4162615594795</v>
       </c>
       <c r="N123" s="11" t="n">
-        <v>29.46550326545543</v>
+        <v>29.60019469099423</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="8" t="inlineStr">
         <is>
-          <t>lap-only (K4 residual steps): every 2025-26 residual step laps at its anniversary</t>
+          <t>base + sub-regional + composition tilt B (EMEA 5 / LatAm 30 / APAC 25) — retired by upgrade 2</t>
         </is>
       </c>
       <c r="C124" s="11" t="n">
-        <v>2.910732193880174</v>
+        <v>2.797413430922292</v>
       </c>
       <c r="D124" s="11" t="n">
-        <v>176.9871287134339</v>
+        <v>176.7930250043633</v>
       </c>
       <c r="E124" s="11" t="n">
-        <v>25.9817104951321</v>
+        <v>25.95321607064054</v>
       </c>
       <c r="F124" s="11" t="n">
-        <v>1.990747787585442</v>
+        <v>2.27299560542554</v>
       </c>
       <c r="G124" s="11" t="n">
-        <v>171.7051486032933</v>
+        <v>172.1779419229572</v>
       </c>
       <c r="H124" s="11" t="n">
-        <v>22.63073858591405</v>
+        <v>22.69305274544576</v>
       </c>
       <c r="I124" s="11" t="n">
-        <v>0.9435507506529328</v>
+        <v>1.84202480617595</v>
       </c>
       <c r="J124" s="11" t="n">
-        <v>187.8933505203212</v>
+        <v>189.5718797508493</v>
       </c>
       <c r="K124" s="11" t="n">
-        <v>31.75773410494469</v>
+        <v>32.04143911548855</v>
       </c>
       <c r="L124" s="11" t="n">
-        <v>1.013196673597509</v>
+        <v>2.510918340989404</v>
       </c>
       <c r="M124" s="11" t="n">
-        <v>184.8071364608028</v>
+        <v>187.5589004803019</v>
       </c>
       <c r="N124" s="11" t="n">
-        <v>29.03320113799212</v>
+        <v>29.46550326545543</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="8" t="inlineStr">
         <is>
-          <t>card v3: last_q residual carry, no lap (card geo)</t>
+          <t>lap-only (K4 residual steps): every 2025-26 residual step laps at its anniversary</t>
         </is>
       </c>
       <c r="C125" s="11" t="n">
-        <v>3.69126637648649</v>
+        <v>2.910732193880174</v>
       </c>
       <c r="D125" s="11" t="n">
-        <v>178.3241057148202</v>
+        <v>176.9871287134339</v>
       </c>
       <c r="E125" s="11" t="n">
-        <v>26.17797871893561</v>
+        <v>25.9817104951321</v>
       </c>
       <c r="F125" s="11" t="n">
-        <v>3.69126637648649</v>
+        <v>1.990747787585442</v>
       </c>
       <c r="G125" s="11" t="n">
-        <v>174.5536872915614</v>
+        <v>171.7051486032933</v>
       </c>
       <c r="H125" s="11" t="n">
-        <v>23.0061759850278</v>
+        <v>22.63073858591405</v>
       </c>
       <c r="I125" s="11" t="n">
-        <v>3.60883637648649</v>
+        <v>0.9435507506529328</v>
       </c>
       <c r="J125" s="11" t="n">
-        <v>192.8726371265034</v>
+        <v>187.8933505203212</v>
       </c>
       <c r="K125" s="11" t="n">
-        <v>32.59933312712161</v>
+        <v>31.75773410494469</v>
       </c>
       <c r="L125" s="11" t="n">
-        <v>3.60883637648649</v>
+        <v>1.013196673597509</v>
       </c>
       <c r="M125" s="11" t="n">
-        <v>189.5761052869207</v>
+        <v>184.8071364608028</v>
       </c>
       <c r="N125" s="11" t="n">
-        <v>29.78240614057524</v>
+        <v>29.03320113799212</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="8" t="inlineStr">
         <is>
-          <t>full lap: ex-NA RNPL sized at the 1H26 residual steps</t>
+          <t>card v3: last_q residual carry, no lap (card geo)</t>
         </is>
       </c>
       <c r="C126" s="11" t="n">
-        <v>3.315947459255554</v>
+        <v>3.69126637648649</v>
       </c>
       <c r="D126" s="11" t="n">
-        <v>177.6812219414954</v>
+        <v>178.3241057148202</v>
       </c>
       <c r="E126" s="11" t="n">
-        <v>26.08360338101152</v>
+        <v>26.17797871893561</v>
       </c>
       <c r="F126" s="11" t="n">
-        <v>2.784074164071932</v>
+        <v>3.69126637648649</v>
       </c>
       <c r="G126" s="11" t="n">
-        <v>173.0340496165458</v>
+        <v>174.5536872915614</v>
       </c>
       <c r="H126" s="11" t="n">
-        <v>22.80588773946074</v>
+        <v>23.0061759850278</v>
       </c>
       <c r="I126" s="11" t="n">
-        <v>1.956877127139422</v>
+        <v>3.60883637648649</v>
       </c>
       <c r="J126" s="11" t="n">
-        <v>189.7864468568733</v>
+        <v>192.8726371265034</v>
       </c>
       <c r="K126" s="11" t="n">
-        <v>32.07770524774872</v>
+        <v>32.59933312712161</v>
       </c>
       <c r="L126" s="11" t="n">
-        <v>1.806523050083998</v>
+        <v>3.60883637648649</v>
       </c>
       <c r="M126" s="11" t="n">
-        <v>186.2647150123214</v>
+        <v>189.5761052869207</v>
       </c>
       <c r="N126" s="11" t="n">
-        <v>29.2621867284357</v>
+        <v>29.78240614057524</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="8" t="inlineStr">
         <is>
-          <t>core mean reversion to the 2023-25 mean</t>
+          <t>full lap: ex-NA RNPL sized at the 1H26 residual steps</t>
         </is>
       </c>
       <c r="C127" s="11" t="n">
-        <v>1.864621082769064</v>
+        <v>3.315947459255554</v>
       </c>
       <c r="D127" s="11" t="n">
-        <v>175.1952449912116</v>
+        <v>177.6812219414954</v>
       </c>
       <c r="E127" s="11" t="n">
-        <v>25.71866196470987</v>
+        <v>26.08360338101152</v>
       </c>
       <c r="F127" s="11" t="n">
-        <v>1.332747787585442</v>
+        <v>2.784074164071932</v>
       </c>
       <c r="G127" s="11" t="n">
-        <v>170.6029328032933</v>
+        <v>173.0340496165458</v>
       </c>
       <c r="H127" s="11" t="n">
-        <v>22.48546654347406</v>
+        <v>22.80588773946074</v>
       </c>
       <c r="I127" s="11" t="n">
-        <v>0.9655507506529332</v>
+        <v>1.956877127139422</v>
       </c>
       <c r="J127" s="11" t="n">
-        <v>187.9344509203212</v>
+        <v>189.7864468568733</v>
       </c>
       <c r="K127" s="11" t="n">
-        <v>31.7646808945527</v>
+        <v>32.07770524774872</v>
       </c>
       <c r="L127" s="11" t="n">
-        <v>1.505196673597509</v>
+        <v>1.806523050083998</v>
       </c>
       <c r="M127" s="11" t="n">
-        <v>185.7110880608028</v>
+        <v>186.2647150123214</v>
       </c>
       <c r="N127" s="11" t="n">
-        <v>29.17521193435212</v>
+        <v>29.2621867284357</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="8" t="inlineStr">
         <is>
-          <t>AR(1) on core (K4 rho 0.747)</t>
+          <t>core mean reversion to the 2023-25 mean</t>
         </is>
       </c>
       <c r="C128" s="11" t="n">
-        <v>3.092067886004471</v>
+        <v>1.864621082769064</v>
       </c>
       <c r="D128" s="11" t="n">
-        <v>177.2977386204736</v>
+        <v>175.1952449912116</v>
       </c>
       <c r="E128" s="11" t="n">
-        <v>26.02730802948552</v>
+        <v>25.71866196470987</v>
       </c>
       <c r="F128" s="11" t="n">
-        <v>2.392956549602292</v>
+        <v>1.332747787585442</v>
       </c>
       <c r="G128" s="11" t="n">
-        <v>172.3788885005477</v>
+        <v>170.6029328032933</v>
       </c>
       <c r="H128" s="11" t="n">
-        <v>22.71953750437219</v>
+        <v>22.48546654347406</v>
       </c>
       <c r="I128" s="11" t="n">
-        <v>1.90083269587952</v>
+        <v>0.9655507506529332</v>
       </c>
       <c r="J128" s="11" t="n">
-        <v>189.6817446503935</v>
+        <v>187.9344509203212</v>
       </c>
       <c r="K128" s="11" t="n">
-        <v>32.06000848080952</v>
+        <v>31.7646808945527</v>
       </c>
       <c r="L128" s="11" t="n">
-        <v>2.347158286681769</v>
+        <v>1.505196673597509</v>
       </c>
       <c r="M128" s="11" t="n">
-        <v>187.2580241325226</v>
+        <v>185.7110880608028</v>
       </c>
       <c r="N128" s="11" t="n">
-        <v>29.41823559121929</v>
+        <v>29.17521193435212</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="8" t="inlineStr">
         <is>
+          <t>AR(1) on core (K4 rho 0.747)</t>
+        </is>
+      </c>
+      <c r="C129" s="11" t="n">
+        <v>3.092067886004471</v>
+      </c>
+      <c r="D129" s="11" t="n">
+        <v>177.2977386204736</v>
+      </c>
+      <c r="E129" s="11" t="n">
+        <v>26.02730802948552</v>
+      </c>
+      <c r="F129" s="11" t="n">
+        <v>2.392956549602292</v>
+      </c>
+      <c r="G129" s="11" t="n">
+        <v>172.3788885005477</v>
+      </c>
+      <c r="H129" s="11" t="n">
+        <v>22.71953750437219</v>
+      </c>
+      <c r="I129" s="11" t="n">
+        <v>1.90083269587952</v>
+      </c>
+      <c r="J129" s="11" t="n">
+        <v>189.6817446503935</v>
+      </c>
+      <c r="K129" s="11" t="n">
+        <v>32.06000848080952</v>
+      </c>
+      <c r="L129" s="11" t="n">
+        <v>2.347158286681769</v>
+      </c>
+      <c r="M129" s="11" t="n">
+        <v>187.2580241325226</v>
+      </c>
+      <c r="N129" s="11" t="n">
+        <v>29.41823559121929</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="8" t="inlineStr">
+        <is>
           <t>base + fee-migration K line (DEC-0008 sensitivity)</t>
         </is>
       </c>
-      <c r="C129" s="11" t="n">
+      <c r="C130" s="11" t="n">
         <v>3.487447459255554</v>
       </c>
-      <c r="D129" s="11" t="n">
+      <c r="D130" s="11" t="n">
         <v>177.9749842914954</v>
       </c>
-      <c r="E129" s="11" t="n">
+      <c r="E130" s="11" t="n">
         <v>26.12672769399152</v>
       </c>
-      <c r="F129" s="11" t="n">
+      <c r="F130" s="11" t="n">
         <v>3.158574164071932</v>
       </c>
-      <c r="G129" s="11" t="n">
+      <c r="G130" s="11" t="n">
         <v>173.6613745665458</v>
       </c>
-      <c r="H129" s="11" t="n">
+      <c r="H130" s="11" t="n">
         <v>22.88856916787073</v>
       </c>
-      <c r="I129" s="11" t="n">
+      <c r="I130" s="11" t="n">
         <v>2.761977127139422</v>
       </c>
-      <c r="J129" s="11" t="n">
+      <c r="J130" s="11" t="n">
         <v>191.2905346768732</v>
       </c>
-      <c r="K129" s="11" t="n">
+      <c r="K130" s="11" t="n">
         <v>32.33192617108512</v>
       </c>
-      <c r="L129" s="11" t="n">
+      <c r="L130" s="11" t="n">
         <v>3.267323050083998</v>
       </c>
-      <c r="M129" s="11" t="n">
+      <c r="M130" s="11" t="n">
         <v>188.9486428523214</v>
       </c>
-      <c r="N129" s="11" t="n">
+      <c r="N130" s="11" t="n">
         <v>29.6838317920997</v>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="8" t="inlineStr">
-        <is>
-          <t>chart helper: ADR $ (printed, then engine)</t>
-        </is>
-      </c>
-      <c r="O132" s="20">
-        <f>O7</f>
-        <v/>
-      </c>
-      <c r="P132" s="20">
-        <f>P7</f>
-        <v/>
-      </c>
-      <c r="Q132" s="20">
-        <f>Q7</f>
-        <v/>
-      </c>
-      <c r="R132" s="20">
-        <f>R7</f>
-        <v/>
-      </c>
-      <c r="S132" s="20">
-        <f>S7</f>
-        <v/>
-      </c>
-      <c r="T132" s="20">
-        <f>T7</f>
-        <v/>
-      </c>
-      <c r="U132" s="20">
-        <f>U7</f>
-        <v/>
-      </c>
-      <c r="V132" s="20">
-        <f>V7</f>
-        <v/>
-      </c>
-      <c r="W132" s="20">
-        <f>W7</f>
-        <v/>
-      </c>
-      <c r="X132" s="20">
-        <f>X7</f>
-        <v/>
-      </c>
-      <c r="Y132" s="20">
-        <f>Y7</f>
-        <v/>
-      </c>
-      <c r="Z132" s="20">
-        <f>Z7</f>
-        <v/>
-      </c>
-      <c r="AA132" s="20">
-        <f>AA7</f>
-        <v/>
-      </c>
-      <c r="AB132" s="20">
-        <f>AB7</f>
-        <v/>
-      </c>
-      <c r="AC132" s="20">
-        <f>AC7</f>
-        <v/>
-      </c>
-      <c r="AD132" s="20">
-        <f>AD7</f>
-        <v/>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="8" t="inlineStr">
         <is>
-          <t>chart helper: Street ADR $</t>
-        </is>
+          <t>chart helper: ADR $ (printed, then engine)</t>
+        </is>
+      </c>
+      <c r="O133" s="20">
+        <f>O7</f>
+        <v/>
+      </c>
+      <c r="P133" s="20">
+        <f>P7</f>
+        <v/>
+      </c>
+      <c r="Q133" s="20">
+        <f>Q7</f>
+        <v/>
+      </c>
+      <c r="R133" s="20">
+        <f>R7</f>
+        <v/>
+      </c>
+      <c r="S133" s="20">
+        <f>S7</f>
+        <v/>
+      </c>
+      <c r="T133" s="20">
+        <f>T7</f>
+        <v/>
+      </c>
+      <c r="U133" s="20">
+        <f>U7</f>
+        <v/>
+      </c>
+      <c r="V133" s="20">
+        <f>V7</f>
+        <v/>
+      </c>
+      <c r="W133" s="20">
+        <f>W7</f>
+        <v/>
+      </c>
+      <c r="X133" s="20">
+        <f>X7</f>
+        <v/>
       </c>
       <c r="Y133" s="20">
-        <f>Y100</f>
+        <f>Y7</f>
         <v/>
       </c>
       <c r="Z133" s="20">
-        <f>Z100</f>
+        <f>Z7</f>
+        <v/>
+      </c>
+      <c r="AA133" s="20">
+        <f>AA7</f>
+        <v/>
+      </c>
+      <c r="AB133" s="20">
+        <f>AB7</f>
+        <v/>
+      </c>
+      <c r="AC133" s="20">
+        <f>AC7</f>
+        <v/>
+      </c>
+      <c r="AD133" s="20">
+        <f>AD7</f>
         <v/>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="8" t="inlineStr">
         <is>
-          <t>chart helper: FX identity (pp)</t>
-        </is>
-      </c>
-      <c r="O134" s="20">
-        <f>O51</f>
-        <v/>
-      </c>
-      <c r="P134" s="20">
-        <f>P51</f>
-        <v/>
-      </c>
-      <c r="Q134" s="20">
-        <f>Q51</f>
-        <v/>
-      </c>
-      <c r="R134" s="20">
-        <f>R51</f>
-        <v/>
-      </c>
-      <c r="S134" s="20">
-        <f>S51</f>
-        <v/>
-      </c>
-      <c r="T134" s="20">
-        <f>T51</f>
-        <v/>
-      </c>
-      <c r="U134" s="20">
-        <f>U51</f>
-        <v/>
-      </c>
-      <c r="V134" s="20">
-        <f>V51</f>
-        <v/>
-      </c>
-      <c r="W134" s="20">
-        <f>W51</f>
-        <v/>
-      </c>
-      <c r="X134" s="20">
-        <f>X51</f>
-        <v/>
+          <t>chart helper: Street ADR $</t>
+        </is>
       </c>
       <c r="Y134" s="20">
-        <f>Y51</f>
+        <f>Y100</f>
         <v/>
       </c>
       <c r="Z134" s="20">
-        <f>Z51</f>
-        <v/>
-      </c>
-      <c r="AA134" s="20">
-        <f>AA51</f>
-        <v/>
-      </c>
-      <c r="AB134" s="20">
-        <f>AB51</f>
-        <v/>
-      </c>
-      <c r="AC134" s="20">
-        <f>AC51</f>
-        <v/>
-      </c>
-      <c r="AD134" s="20">
-        <f>AD51</f>
+        <f>Z100</f>
         <v/>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="8" t="inlineStr">
         <is>
+          <t>chart helper: FX identity (pp)</t>
+        </is>
+      </c>
+      <c r="O135" s="20">
+        <f>O51</f>
+        <v/>
+      </c>
+      <c r="P135" s="20">
+        <f>P51</f>
+        <v/>
+      </c>
+      <c r="Q135" s="20">
+        <f>Q51</f>
+        <v/>
+      </c>
+      <c r="R135" s="20">
+        <f>R51</f>
+        <v/>
+      </c>
+      <c r="S135" s="20">
+        <f>S51</f>
+        <v/>
+      </c>
+      <c r="T135" s="20">
+        <f>T51</f>
+        <v/>
+      </c>
+      <c r="U135" s="20">
+        <f>U51</f>
+        <v/>
+      </c>
+      <c r="V135" s="20">
+        <f>V51</f>
+        <v/>
+      </c>
+      <c r="W135" s="20">
+        <f>W51</f>
+        <v/>
+      </c>
+      <c r="X135" s="20">
+        <f>X51</f>
+        <v/>
+      </c>
+      <c r="Y135" s="20">
+        <f>Y51</f>
+        <v/>
+      </c>
+      <c r="Z135" s="20">
+        <f>Z51</f>
+        <v/>
+      </c>
+      <c r="AA135" s="20">
+        <f>AA51</f>
+        <v/>
+      </c>
+      <c r="AB135" s="20">
+        <f>AB51</f>
+        <v/>
+      </c>
+      <c r="AC135" s="20">
+        <f>AC51</f>
+        <v/>
+      </c>
+      <c r="AD135" s="20">
+        <f>AD51</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="8" t="inlineStr">
+        <is>
           <t>chart helper: disclosed FX (pp)</t>
         </is>
       </c>
-      <c r="O135" s="20">
+      <c r="O136" s="20">
         <f>O10</f>
         <v/>
       </c>
-      <c r="P135" s="20">
+      <c r="P136" s="20">
         <f>P10</f>
         <v/>
       </c>
-      <c r="Q135" s="20">
+      <c r="Q136" s="20">
         <f>Q10</f>
         <v/>
       </c>
-      <c r="R135" s="20">
+      <c r="R136" s="20">
         <f>R10</f>
         <v/>
       </c>
-      <c r="S135" s="20">
+      <c r="S136" s="20">
         <f>S10</f>
         <v/>
       </c>
-      <c r="T135" s="20">
+      <c r="T136" s="20">
         <f>T10</f>
         <v/>
       </c>
-      <c r="U135" s="20">
+      <c r="U136" s="20">
         <f>U10</f>
         <v/>
       </c>
-      <c r="V135" s="20">
+      <c r="V136" s="20">
         <f>V10</f>
         <v/>
       </c>
-      <c r="W135" s="20">
+      <c r="W136" s="20">
         <f>W10</f>
         <v/>
       </c>
-      <c r="X135" s="20">
+      <c r="X136" s="20">
         <f>X10</f>
         <v/>
       </c>

</xml_diff>